<commit_message>
Update index: 5997 → 6035 [scan complete - 5 new businesses found]
Scanned דרך בית לחם 135 through 98 (indices 5997-6034).
Found 5 new businesses:
- פרליני-שוקולד בלגי משובח (37)
- יוחנן בארי-שירי פרידמן / אדריכלות (37)
- בית ספר לנהיגה הבירה (71)
- לוי רפי / מורה לנהיגה (71)
- עם רם הנדסה / שיפוצים (98)
</commit_message>
<xml_diff>
--- a/excel outputs/דוח נכסים לתאריך:25-07-2026.xlsx
+++ b/excel outputs/דוח נכסים לתאריך:25-07-2026.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ממצאים" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="נכסים חשודים" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,23 +26,19 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Arial"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Arial"/>
       <color rgb="000563C1"/>
-      <sz val="10"/>
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -62,6 +58,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -91,10 +92,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -106,6 +107,12 @@
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -473,13 +480,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="42" customWidth="1" min="5" max="5"/>
     <col width="42" customWidth="1" min="6" max="6"/>
     <col width="42" customWidth="1" min="7" max="7"/>
@@ -548,8 +555,8 @@
           <t>https://www.d.co.il/80254982/40030057/</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
@@ -577,8 +584,8 @@
           <t>https://www.d.co.il/80095883/19745/</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr"/>
-      <c r="G3" s="4" t="inlineStr"/>
+      <c r="F3" s="4" t="n"/>
+      <c r="G3" s="4" t="n"/>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -606,8 +613,8 @@
           <t>https://www.d.co.il/74082710/40030024/</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -635,16 +642,155 @@
           <t>https://www.d.co.il/80337849/13110/</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr"/>
-      <c r="G5" s="4" t="inlineStr"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="n"/>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>פרליני-שוקולד בלגי משובח</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>דרך בית לחם 37, ירושלים</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>ייצור, יבוא ושיווק שוקולד</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80061203/9010047/</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>יוחנן בארי-שירי פרידמן</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>דרך בית לחם 37, ירושלים</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>אדריכלים ומשרדי אדריכלות ✅</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/77255750/630/</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="n"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>בית ספר לנהיגה הבירה</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>דרך בית לחם 71, ירושלים</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>בית ספר לנהיגה</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80015970/8450/</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2" t="n"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>לוי רפי</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>דרך בית לחם 71, ירושלים</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>מורה לנהיגה</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/74834980/8450/</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="n"/>
+      <c r="G9" s="4" t="n"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>עם רם הנדסה</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>דרך בית לחם 98, ירושלים</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>שיפוצים ותיקונים</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80309256/48570/</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2" t="n"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Excel report: 19 businesses total (25-07-2026)
</commit_message>
<xml_diff>
--- a/excel outputs/דוח נכסים לתאריך:25-07-2026.xlsx
+++ b/excel outputs/דוח נכסים לתאריך:25-07-2026.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="נכסים חשודים" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="נכסים" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,12 +33,8 @@
     <font>
       <sz val="10"/>
     </font>
-    <font>
-      <color rgb="000563C1"/>
-      <u val="single"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -60,11 +56,6 @@
         <fgColor rgb="00D6E4F0"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -76,43 +67,31 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="001F4E79"/>
+        <color rgb="00AAAAAA"/>
       </left>
       <right style="thin">
-        <color rgb="001F4E79"/>
+        <color rgb="00AAAAAA"/>
       </right>
       <top style="thin">
-        <color rgb="001F4E79"/>
+        <color rgb="00AAAAAA"/>
       </top>
       <bottom style="thin">
-        <color rgb="001F4E79"/>
+        <color rgb="00AAAAAA"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -480,19 +459,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25" customHeight="1">
+    <row r="1" ht="20" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>שם העסק</t>
@@ -529,7 +508,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="20" customHeight="1">
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>ירון מרגולין</t>
@@ -550,7 +529,7 @@
           <t>גבוה</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>https://www.d.co.il/80254982/40030057/</t>
         </is>
@@ -558,36 +537,36 @@
       <c r="F2" s="2" t="n"/>
       <c r="G2" s="2" t="n"/>
     </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>שפיז משה - עובד סוציאלי</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>דרך בית לחם 106, ירושלים</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>ייעוץ וטיפול - אישי, זוגי ומשפחתי</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>https://www.d.co.il/80095883/19745/</t>
         </is>
       </c>
-      <c r="F3" s="4" t="n"/>
-      <c r="G3" s="4" t="n"/>
-    </row>
-    <row r="4" ht="20" customHeight="1">
+      <c r="F3" s="3" t="n"/>
+      <c r="G3" s="3" t="n"/>
+    </row>
+    <row r="4" ht="18" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>סאלמה משה</t>
@@ -608,7 +587,7 @@
           <t>גבוה</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>https://www.d.co.il/74082710/40030024/</t>
         </is>
@@ -616,36 +595,36 @@
       <c r="F4" s="2" t="n"/>
       <c r="G4" s="2" t="n"/>
     </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>מר מדביר</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>דרך בית לחם 125, ירושלים</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>הדברת מזיקים</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>https://www.d.co.il/80337849/13110/</t>
         </is>
       </c>
-      <c r="F5" s="4" t="n"/>
-      <c r="G5" s="4" t="n"/>
-    </row>
-    <row r="6" ht="20" customHeight="1">
+      <c r="F5" s="3" t="n"/>
+      <c r="G5" s="3" t="n"/>
+    </row>
+    <row r="6" ht="18" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>פרליני-שוקולד בלגי משובח</t>
@@ -666,7 +645,7 @@
           <t>גבוה</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>https://www.d.co.il/80061203/9010047/</t>
         </is>
@@ -674,36 +653,36 @@
       <c r="F6" s="2" t="n"/>
       <c r="G6" s="2" t="n"/>
     </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>יוחנן בארי-שירי פרידמן</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>דרך בית לחם 37, ירושלים</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>אדריכלים ומשרדי אדריכלות ✅</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>אדריכלים ומשרדי אדריכלות</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>https://www.d.co.il/77255750/630/</t>
         </is>
       </c>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="n"/>
-    </row>
-    <row r="8" ht="20" customHeight="1">
+      <c r="F7" s="3" t="n"/>
+      <c r="G7" s="3" t="n"/>
+    </row>
+    <row r="8" ht="18" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>בית ספר לנהיגה הבירה</t>
@@ -724,7 +703,7 @@
           <t>גבוה</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>https://www.d.co.il/80015970/8450/</t>
         </is>
@@ -732,36 +711,36 @@
       <c r="F8" s="2" t="n"/>
       <c r="G8" s="2" t="n"/>
     </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>לוי רפי</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>דרך בית לחם 71, ירושלים</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>מורה לנהיגה</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>https://www.d.co.il/74834980/8450/</t>
         </is>
       </c>
-      <c r="F9" s="4" t="n"/>
-      <c r="G9" s="4" t="n"/>
-    </row>
-    <row r="10" ht="20" customHeight="1">
+      <c r="F9" s="3" t="n"/>
+      <c r="G9" s="3" t="n"/>
+    </row>
+    <row r="10" ht="18" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>עם רם הנדסה</t>
@@ -782,13 +761,303 @@
           <t>גבוה</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>https://www.d.co.il/80309256/48570/</t>
         </is>
       </c>
       <c r="F10" s="2" t="n"/>
       <c r="G10" s="2" t="n"/>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>כוכב ירושלים-עבודות עפר ופיתוח בע"מ</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>דרך ג'בל מוכבר 42, ירושלים</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>עבודות עפר ופיתוח / פינוי פסולת</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80272515/40210/</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="n"/>
+      <c r="G11" s="3" t="n"/>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>אחים אבו חאמד לעבודות עפר ופיתוח בע"מ</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>דרך ג'בל מוכבר 73, ירושלים</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>עבודות עפר ופיתוח</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80158703/37290/</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="n"/>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>רפאל יונתן לאוס</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>דרך האחיות 12, ירושלים</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>פסיכולוגים קליניים</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80223646/40270/</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="n"/>
+      <c r="G13" s="3" t="n"/>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>הבית של גילה</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>דרך האחיות 27, ירושלים</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>צימרים ולינה כפרית</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80125598/7494/</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n"/>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>קרן יוחנן</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>דרך האילנות 7, ירושלים</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>לימודי ריקוד ותנועה</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80146556/8560/</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="n"/>
+      <c r="G15" s="3" t="n"/>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>המנסרים ביהלום בע"מ</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>דרך החורש 2, ירושלים</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>ניסור וקידוח בטון</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80048762/5480/</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>ברסקו שופ בע"מ</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>דרך החורש 12, ירושלים</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>סוללות, מטענים וספקי כוח</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80224236/35580/</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="n"/>
+      <c r="G17" s="3" t="n"/>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>דגנית-נטורופתית מוסמכת</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>דרך החורש 12, ירושלים</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>נטורופתיה / רפואה אלטרנטיבית</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80107497/40030002/</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="n"/>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>נטלי קוסמטיקה</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>דרך החורש 4, ירושלים</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>עיצוב גבות / קוסמטיקה</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80194653/38143/</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="n"/>
+      <c r="G19" s="3" t="n"/>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>עו"ד ונוטריון יאיר משה</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>דרך החורש 15, ירושלים</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>עורכי דין / נוטריון</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/64558930/38010/</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Excel report: 26 businesses total (25-07-2026)
</commit_message>
<xml_diff>
--- a/excel outputs/דוח נכסים לתאריך:25-07-2026.xlsx
+++ b/excel outputs/דוח נכסים לתאריך:25-07-2026.xlsx
@@ -57,7 +57,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -79,11 +79,17 @@
         <color rgb="00AAAAAA"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -93,6 +99,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -459,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1059,6 +1071,209 @@
       <c r="F20" s="2" t="n"/>
       <c r="G20" s="2" t="n"/>
     </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>יוני אלקינס - EMDR</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>דרך חברון 37, ירושלים</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>עובד סוציאלי</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80275352/9010019/</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr"/>
+      <c r="G21" s="4" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>עוז לוי</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>דרך חברון 46, ירושלים</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>רפואה סינית</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80037906/40030001/</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr"/>
+      <c r="G22" s="5" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>קייטרינג מליסה</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>דרך חברון 46, ירושלים</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>קייטרינג</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80064419/44380/</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr"/>
+      <c r="G23" s="4" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>גד תשתיות ופיתוח בע"מ</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>דרך חברון 110, ירושלים</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>עבודות עפר ופיתוח</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/62246610/37290/</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr"/>
+      <c r="G24" s="5" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>אביטל-עיסויים ורפואה אלטרנטיבית-לנשים בלבד!</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>דרך חברון 117, ירושלים</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>רפואה משלימה</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80234602/40030057/</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr"/>
+      <c r="G25" s="4" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>אמויאל איציק</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>דרך חברון 150, ירושלים</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>DJ ומוזיקה לאירועים</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/30976070/24390/</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr"/>
+      <c r="G26" s="5" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>דואר ישראל</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>דרך יריחו 207, ירושלים</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>שירותי דואר</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80307506/11820/</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr"/>
+      <c r="G27" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>